<commit_message>
Added new cybercrime case
</commit_message>
<xml_diff>
--- a/Cyberlaw_Women_India_Verified_2024_2026.xlsx
+++ b/Cyberlaw_Women_India_Verified_2024_2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/81ace244192e6b05/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/81ace244192e6b05/Desktop/RP1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="62" documentId="8_{299B988A-799C-4FE1-AAF1-D9AC11FEDE7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF780997-394B-44A0-9CCB-00C1FDDD093F}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="8_{9C277E61-18F4-4A77-BA5F-BA24AA7734D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{847AAAD2-63F0-484A-BEED-C6FC6C588D52}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="207">
   <si>
     <t>case_id</t>
   </si>
@@ -651,6 +651,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.mha.gov.in/MHA1/Par2017/pdfs/par2024-pdfs/LS06082024/2504.pdf </t>
+  </si>
+  <si>
+    <t>P-33</t>
   </si>
 </sst>
 </file>
@@ -1074,7 +1077,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P33"/>
+  <dimension ref="A1:P34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1178,7 +1181,7 @@
         <v>1840</v>
       </c>
       <c r="L2" s="3">
-        <f t="shared" ref="L2:L33" si="0">K2/I2*100</f>
+        <f t="shared" ref="L2:L34" si="0">K2/I2*100</f>
         <v>4.2012009955019742</v>
       </c>
       <c r="M2" s="2" t="s">
@@ -2775,40 +2778,92 @@
         <v>190</v>
       </c>
     </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A34" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="B34">
+        <v>2025</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="G34" t="s">
+        <v>189</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I34" s="4">
+        <v>3300</v>
+      </c>
+      <c r="J34" s="4">
+        <v>240</v>
+      </c>
+      <c r="K34" s="2">
+        <v>21</v>
+      </c>
+      <c r="L34" s="3">
+        <f t="shared" si="0"/>
+        <v>0.63636363636363635</v>
+      </c>
+      <c r="M34" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="N34" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="O34" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="P34" s="11" t="s">
+        <v>190</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="P32" r:id="rId1" xr:uid="{3AF25670-4CEB-49CD-BA5E-CBCD0BD00BCF}"/>
-    <hyperlink ref="P33" r:id="rId2" xr:uid="{B47D01DE-7B71-41BC-965C-8257659FE0EC}"/>
-    <hyperlink ref="P31" r:id="rId3" xr:uid="{14D62B01-4985-4489-8899-D29F9A707642}"/>
-    <hyperlink ref="P30" r:id="rId4" xr:uid="{DC43A5A4-146A-42EC-A693-84AA400DAAC6}"/>
-    <hyperlink ref="P29" r:id="rId5" xr:uid="{CC876FA8-6EC8-40FD-963F-DC6E91ACAFC2}"/>
-    <hyperlink ref="P28" r:id="rId6" xr:uid="{BCF76780-E613-4D0C-BD0F-47DD47926653}"/>
-    <hyperlink ref="P27" r:id="rId7" xr:uid="{98299004-A85A-4474-9D8A-6A5BB1C6C5E9}"/>
-    <hyperlink ref="P26" r:id="rId8" xr:uid="{7735B20B-6B79-4E7D-9F34-E576C5364857}"/>
-    <hyperlink ref="P25" r:id="rId9" xr:uid="{09E3E98A-26EF-4D8D-9A8D-84F93EC38590}"/>
-    <hyperlink ref="P24" r:id="rId10" xr:uid="{45FE6F93-EB62-4CBF-AD6A-863CD784F354}"/>
-    <hyperlink ref="P23" r:id="rId11" xr:uid="{F5C1471E-CE84-4C71-93E9-1528B97D5CA9}"/>
-    <hyperlink ref="P22" r:id="rId12" xr:uid="{C18DA440-EE35-4776-B250-22EDD55687E7}"/>
-    <hyperlink ref="P21" r:id="rId13" xr:uid="{225FBB8E-4262-46B7-ABAE-90D7900A026B}"/>
-    <hyperlink ref="P20" r:id="rId14" xr:uid="{2AA3A727-7D2D-492F-B9AA-066EE1BB613D}"/>
-    <hyperlink ref="P19" r:id="rId15" xr:uid="{7D6FDBD5-8362-4D43-970F-CB0C87A84CE8}"/>
-    <hyperlink ref="P18" r:id="rId16" xr:uid="{80DD1F25-1560-4401-8116-F4BEFBF7BD35}"/>
-    <hyperlink ref="P17" r:id="rId17" xr:uid="{E45218EC-887E-46B3-8FFC-4CED6E0662FF}"/>
-    <hyperlink ref="P16" r:id="rId18" xr:uid="{FED8C43D-52E8-402F-9388-3915D0B8443A}"/>
-    <hyperlink ref="P15" r:id="rId19" xr:uid="{C26B7A0A-7410-4A84-8DC3-AA7CBB74A0C3}"/>
-    <hyperlink ref="P14" r:id="rId20" xr:uid="{B1E527EB-88B6-4280-822C-B8AD36BA293F}"/>
-    <hyperlink ref="P13" r:id="rId21" xr:uid="{A98109EC-FDAC-4FEB-81F0-30463F9E26A4}"/>
-    <hyperlink ref="P12" r:id="rId22" xr:uid="{7F427CB6-9A6B-4DC3-84BB-093EE59DD791}"/>
-    <hyperlink ref="P11" r:id="rId23" xr:uid="{EDCFD420-60D8-4D4A-9C2B-7E119993912D}"/>
-    <hyperlink ref="P10" r:id="rId24" xr:uid="{B363CECC-A49A-48D9-9EF8-8778FD52503B}"/>
-    <hyperlink ref="P9" r:id="rId25" xr:uid="{0AEED889-DA96-429E-8ADB-578778A40CD5}"/>
-    <hyperlink ref="P8" r:id="rId26" xr:uid="{A6855E54-0B50-4933-BD22-1C4A24D76270}"/>
-    <hyperlink ref="P7" r:id="rId27" xr:uid="{E08A5264-E973-40CE-86DC-10178D48A6FE}"/>
-    <hyperlink ref="P6" r:id="rId28" xr:uid="{3C981E66-AAE8-4475-B755-4E51D1350B89}"/>
-    <hyperlink ref="P5" r:id="rId29" xr:uid="{9E62481F-4B60-487A-9A63-F910F33C5533}"/>
-    <hyperlink ref="P4" r:id="rId30" xr:uid="{1A911014-5FE3-430E-A5E0-2459E7453C10}"/>
-    <hyperlink ref="P3" r:id="rId31" xr:uid="{148705B5-CAD8-4A85-9E1A-F05EAC793000}"/>
-    <hyperlink ref="P2" r:id="rId32" xr:uid="{1E6481F5-5541-4A0D-BC19-F9C89A50591D}"/>
+    <hyperlink ref="P31" r:id="rId2" xr:uid="{14D62B01-4985-4489-8899-D29F9A707642}"/>
+    <hyperlink ref="P30" r:id="rId3" xr:uid="{DC43A5A4-146A-42EC-A693-84AA400DAAC6}"/>
+    <hyperlink ref="P29" r:id="rId4" xr:uid="{CC876FA8-6EC8-40FD-963F-DC6E91ACAFC2}"/>
+    <hyperlink ref="P28" r:id="rId5" xr:uid="{BCF76780-E613-4D0C-BD0F-47DD47926653}"/>
+    <hyperlink ref="P27" r:id="rId6" xr:uid="{98299004-A85A-4474-9D8A-6A5BB1C6C5E9}"/>
+    <hyperlink ref="P26" r:id="rId7" xr:uid="{7735B20B-6B79-4E7D-9F34-E576C5364857}"/>
+    <hyperlink ref="P25" r:id="rId8" xr:uid="{09E3E98A-26EF-4D8D-9A8D-84F93EC38590}"/>
+    <hyperlink ref="P24" r:id="rId9" xr:uid="{45FE6F93-EB62-4CBF-AD6A-863CD784F354}"/>
+    <hyperlink ref="P23" r:id="rId10" xr:uid="{F5C1471E-CE84-4C71-93E9-1528B97D5CA9}"/>
+    <hyperlink ref="P22" r:id="rId11" xr:uid="{C18DA440-EE35-4776-B250-22EDD55687E7}"/>
+    <hyperlink ref="P21" r:id="rId12" xr:uid="{225FBB8E-4262-46B7-ABAE-90D7900A026B}"/>
+    <hyperlink ref="P20" r:id="rId13" xr:uid="{2AA3A727-7D2D-492F-B9AA-066EE1BB613D}"/>
+    <hyperlink ref="P19" r:id="rId14" xr:uid="{7D6FDBD5-8362-4D43-970F-CB0C87A84CE8}"/>
+    <hyperlink ref="P18" r:id="rId15" xr:uid="{80DD1F25-1560-4401-8116-F4BEFBF7BD35}"/>
+    <hyperlink ref="P17" r:id="rId16" xr:uid="{E45218EC-887E-46B3-8FFC-4CED6E0662FF}"/>
+    <hyperlink ref="P16" r:id="rId17" xr:uid="{FED8C43D-52E8-402F-9388-3915D0B8443A}"/>
+    <hyperlink ref="P15" r:id="rId18" xr:uid="{C26B7A0A-7410-4A84-8DC3-AA7CBB74A0C3}"/>
+    <hyperlink ref="P14" r:id="rId19" xr:uid="{B1E527EB-88B6-4280-822C-B8AD36BA293F}"/>
+    <hyperlink ref="P13" r:id="rId20" xr:uid="{A98109EC-FDAC-4FEB-81F0-30463F9E26A4}"/>
+    <hyperlink ref="P12" r:id="rId21" xr:uid="{7F427CB6-9A6B-4DC3-84BB-093EE59DD791}"/>
+    <hyperlink ref="P11" r:id="rId22" xr:uid="{EDCFD420-60D8-4D4A-9C2B-7E119993912D}"/>
+    <hyperlink ref="P10" r:id="rId23" xr:uid="{B363CECC-A49A-48D9-9EF8-8778FD52503B}"/>
+    <hyperlink ref="P9" r:id="rId24" xr:uid="{0AEED889-DA96-429E-8ADB-578778A40CD5}"/>
+    <hyperlink ref="P8" r:id="rId25" xr:uid="{A6855E54-0B50-4933-BD22-1C4A24D76270}"/>
+    <hyperlink ref="P7" r:id="rId26" xr:uid="{E08A5264-E973-40CE-86DC-10178D48A6FE}"/>
+    <hyperlink ref="P6" r:id="rId27" xr:uid="{3C981E66-AAE8-4475-B755-4E51D1350B89}"/>
+    <hyperlink ref="P5" r:id="rId28" xr:uid="{9E62481F-4B60-487A-9A63-F910F33C5533}"/>
+    <hyperlink ref="P4" r:id="rId29" xr:uid="{1A911014-5FE3-430E-A5E0-2459E7453C10}"/>
+    <hyperlink ref="P3" r:id="rId30" xr:uid="{148705B5-CAD8-4A85-9E1A-F05EAC793000}"/>
+    <hyperlink ref="P2" r:id="rId31" xr:uid="{1E6481F5-5541-4A0D-BC19-F9C89A50591D}"/>
+    <hyperlink ref="P33" r:id="rId32" xr:uid="{B47D01DE-7B71-41BC-965C-8257659FE0EC}"/>
+    <hyperlink ref="P34" r:id="rId33" xr:uid="{352BEF4F-5799-41EC-8CA9-AD99E236152A}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Deleted a cybercrime case
</commit_message>
<xml_diff>
--- a/Cyberlaw_Women_India_Verified_2024_2026.xlsx
+++ b/Cyberlaw_Women_India_Verified_2024_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/81ace244192e6b05/Desktop/RP1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{9C277E61-18F4-4A77-BA5F-BA24AA7734D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{847AAAD2-63F0-484A-BEED-C6FC6C588D52}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{D27E04FA-C659-495A-8369-529608D967EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{403B610C-CDCC-4CB0-9A30-6A542584A8DE}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="206">
   <si>
     <t>case_id</t>
   </si>
@@ -651,9 +651,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.mha.gov.in/MHA1/Par2017/pdfs/par2024-pdfs/LS06082024/2504.pdf </t>
-  </si>
-  <si>
-    <t>P-33</t>
   </si>
 </sst>
 </file>
@@ -2779,55 +2776,20 @@
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A34" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="B34">
-        <v>2025</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="E34" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="F34" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="G34" t="s">
-        <v>189</v>
-      </c>
-      <c r="H34" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="I34" s="4">
-        <v>3300</v>
-      </c>
-      <c r="J34" s="4">
-        <v>240</v>
-      </c>
-      <c r="K34" s="2">
-        <v>21</v>
-      </c>
-      <c r="L34" s="3">
-        <f t="shared" si="0"/>
-        <v>0.63636363636363635</v>
-      </c>
-      <c r="M34" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="N34" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="O34" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="P34" s="11" t="s">
-        <v>190</v>
-      </c>
+      <c r="A34" s="2"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+      <c r="H34" s="4"/>
+      <c r="I34" s="4"/>
+      <c r="J34" s="4"/>
+      <c r="K34" s="2"/>
+      <c r="L34" s="3"/>
+      <c r="M34" s="4"/>
+      <c r="N34" s="4"/>
+      <c r="O34" s="4"/>
+      <c r="P34" s="11"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2863,7 +2825,6 @@
     <hyperlink ref="P3" r:id="rId30" xr:uid="{148705B5-CAD8-4A85-9E1A-F05EAC793000}"/>
     <hyperlink ref="P2" r:id="rId31" xr:uid="{1E6481F5-5541-4A0D-BC19-F9C89A50591D}"/>
     <hyperlink ref="P33" r:id="rId32" xr:uid="{B47D01DE-7B71-41BC-965C-8257659FE0EC}"/>
-    <hyperlink ref="P34" r:id="rId33" xr:uid="{352BEF4F-5799-41EC-8CA9-AD99E236152A}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>